<commit_message>
Simplify date requirements for v1
</commit_message>
<xml_diff>
--- a/src/lib/content/2024-10-01 Campus Collaboration Living Bibliography.xlsx
+++ b/src/lib/content/2024-10-01 Campus Collaboration Living Bibliography.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mhal9222/Desktop/living-bibliography/src/lib/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{016D10E7-F5A3-B94F-BE63-AD78CE4DA2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A06F0A-3CFE-304D-B0DD-2DD87C932B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{62C1BFAF-8520-5D4C-BFE9-88B66F49E369}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{62C1BFAF-8520-5D4C-BFE9-88B66F49E369}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="194">
   <si>
     <t>A living bibliography</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Publisher</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
     <t>Annotation</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
   </si>
   <si>
     <t>Link</t>
-  </si>
-  <si>
-    <t>Date added to bibliography</t>
   </si>
   <si>
     <t>Latitude</t>
@@ -651,6 +645,9 @@
   </si>
   <si>
     <t>campus-collaboration</t>
+  </si>
+  <si>
+    <t>Date updated</t>
   </si>
 </sst>
 </file>
@@ -1167,12 +1164,20 @@
         <v>6</v>
       </c>
     </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="1">
+        <v>45566</v>
+      </c>
+    </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1185,38 +1190,37 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6608C388-4639-4F4E-9326-DC48CED4E1B6}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="42.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="43.7109375" customWidth="1"/>
-    <col min="6" max="6" width="99" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
-    <col min="10" max="10" width="42.7109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="25.42578125" customWidth="1"/>
+    <col min="3" max="3" width="42.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" customWidth="1"/>
+    <col min="5" max="5" width="99" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" customWidth="1"/>
+    <col min="8" max="8" width="42.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17">
+    <row r="1" spans="1:9" ht="17">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E1" s="6" t="s">
@@ -1228,764 +1232,590 @@
       <c r="G1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="8"/>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:9" ht="170">
+      <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="B2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11" ht="170">
-      <c r="A2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="E2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="10">
+        <v>-37.913798892611098</v>
+      </c>
+      <c r="G2" s="11">
+        <v>145.138632494722</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="102">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>-33.810661633039601</v>
+      </c>
+      <c r="G3">
+        <v>151.028741704049</v>
+      </c>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="153">
+      <c r="A4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>-37.798227185013197</v>
+      </c>
+      <c r="G4">
+        <v>144.96137096393301</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="68">
+      <c r="A5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5">
+        <v>-33.888261572671198</v>
+      </c>
+      <c r="G5">
+        <v>151.18642147408201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="119">
+      <c r="A6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6">
+        <v>38.033679630343499</v>
+      </c>
+      <c r="G6">
+        <v>-78.507183269423606</v>
+      </c>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" ht="102">
+      <c r="A7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7">
+        <v>38.033679630343499</v>
+      </c>
+      <c r="G7">
+        <v>-78.507183269423606</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="136">
+      <c r="A8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8">
+        <v>42.371358419161901</v>
+      </c>
+      <c r="G8">
+        <v>-71.121215603410306</v>
+      </c>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:9" ht="136">
+      <c r="A9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9">
+        <v>42.371875034443001</v>
+      </c>
+      <c r="G9">
+        <v>-71.118086827892697</v>
+      </c>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" ht="102">
+      <c r="A10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10">
+        <v>36.001547287548</v>
+      </c>
+      <c r="G10">
+        <v>-78.937745805743205</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="153">
+      <c r="A11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11">
+        <v>41.787806146843899</v>
+      </c>
+      <c r="G11">
+        <v>-87.597806297506594</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="153">
+      <c r="A12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12">
+        <v>37.870278012646096</v>
+      </c>
+      <c r="G12">
+        <v>-122.25893489032801</v>
+      </c>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" ht="136">
+      <c r="A13" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="136">
+      <c r="A14" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="136">
+      <c r="A15" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" ht="102">
+      <c r="A16" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1">
-        <v>45453</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H2" s="10">
-        <v>-37.913798892611098</v>
-      </c>
-      <c r="I2" s="11">
-        <v>145.138632494722</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="102">
-      <c r="A3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45454</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H3">
-        <v>-33.810661633039601</v>
-      </c>
-      <c r="I3">
-        <v>151.028741704049</v>
-      </c>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="153">
-      <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45455</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H4">
-        <v>-37.798227185013197</v>
-      </c>
-      <c r="I4">
-        <v>144.96137096393301</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="68">
-      <c r="A5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="E16" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="102">
+      <c r="A17" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="85">
+      <c r="A18" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="1:9" ht="68">
+      <c r="A19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="68">
+      <c r="A20" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="68">
+      <c r="A21" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" ht="68">
+      <c r="A22" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="85">
+      <c r="A23" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="85">
+      <c r="A24" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" ht="136">
+      <c r="A25" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="1">
-        <v>45456</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H5">
-        <v>-33.888261572671198</v>
-      </c>
-      <c r="I5">
-        <v>151.18642147408201</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="119">
-      <c r="A6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="1">
-        <v>45457</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H6">
-        <v>38.033679630343499</v>
-      </c>
-      <c r="I6">
-        <v>-78.507183269423606</v>
-      </c>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" ht="102">
-      <c r="A7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="1">
-        <v>45458</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H7">
-        <v>38.033679630343499</v>
-      </c>
-      <c r="I7">
-        <v>-78.507183269423606</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="136">
-      <c r="A8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="1">
-        <v>45459</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G8" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H8">
-        <v>42.371358419161901</v>
-      </c>
-      <c r="I8">
-        <v>-71.121215603410306</v>
-      </c>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" ht="136">
-      <c r="A9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="1">
-        <v>45460</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H9">
-        <v>42.371875034443001</v>
-      </c>
-      <c r="I9">
-        <v>-71.118086827892697</v>
-      </c>
-      <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" ht="102">
-      <c r="A10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="E25" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="68">
+      <c r="A26" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="119">
+      <c r="A27" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="119">
+      <c r="A28" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="1">
-        <v>45461</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H10">
-        <v>36.001547287548</v>
-      </c>
-      <c r="I10">
-        <v>-78.937745805743205</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="153">
-      <c r="A11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="1">
-        <v>45462</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G11" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H11">
-        <v>41.787806146843899</v>
-      </c>
-      <c r="I11">
-        <v>-87.597806297506594</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="153">
-      <c r="A12" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="1">
-        <v>45463</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G12" s="1">
-        <v>45545</v>
-      </c>
-      <c r="H12">
-        <v>37.870278012646096</v>
-      </c>
-      <c r="I12">
-        <v>-122.25893489032801</v>
-      </c>
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" ht="136">
-      <c r="A13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="1">
-        <v>45464</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="136">
-      <c r="A14" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="1">
-        <v>45465</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="136">
-      <c r="A15" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="1">
-        <v>45466</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="1">
-        <v>45545</v>
-      </c>
-      <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" ht="102">
-      <c r="A16" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="1">
-        <v>45467</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G16" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="102">
-      <c r="A17" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="1">
-        <v>45468</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G17" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="85">
-      <c r="A18" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C18" s="1">
-        <v>45469</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="1">
-        <v>45545</v>
-      </c>
-      <c r="K18" s="3"/>
-    </row>
-    <row r="19" spans="1:11" ht="68">
-      <c r="A19" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="1">
-        <v>45470</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="G19" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="68">
-      <c r="A20" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C20" s="1">
-        <v>45471</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G20" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="68">
-      <c r="A21" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="1">
-        <v>45472</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="G21" s="1">
-        <v>45545</v>
-      </c>
-      <c r="K21" s="3"/>
-    </row>
-    <row r="22" spans="1:11" ht="68">
-      <c r="A22" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C22" s="1">
-        <v>45473</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="G22" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="85">
-      <c r="A23" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C23" s="1">
-        <v>45474</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G23" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="85">
-      <c r="A24" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C24" s="1">
-        <v>45475</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="G24" s="1">
-        <v>45545</v>
-      </c>
-      <c r="K24" s="3"/>
-    </row>
-    <row r="25" spans="1:11" ht="136">
-      <c r="A25" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="1">
-        <v>45476</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="G25" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="68">
-      <c r="A26" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C26" s="1">
-        <v>45477</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="G26" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="119">
-      <c r="A27" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" s="1">
-        <v>45478</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="G27" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="119">
-      <c r="A28" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B28" s="3" t="s">
+      <c r="E28" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C28" s="1">
-        <v>45479</v>
-      </c>
-      <c r="D28" s="3" t="s">
+    </row>
+    <row r="29" spans="1:9" ht="102">
+      <c r="A29" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F28" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="G28" s="1">
-        <v>45545</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="102">
-      <c r="A29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="D29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>133</v>
-      </c>
-      <c r="C29" s="1">
-        <v>45480</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="G29" s="1">
-        <v>45545</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{C2E11FBC-70C3-4175-B407-3AE3B5AB88B9}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{5D46BCE6-875C-4DD1-A561-F12602AA0818}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{C9298B6A-3400-4298-BFA1-CDF2C509364B}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{BBEFC72C-BD5C-40B9-99D1-E240C18CA4E6}"/>
-    <hyperlink ref="F6" r:id="rId5" xr:uid="{63ED79AB-A47C-4E8A-AE04-F860DCF5B935}"/>
-    <hyperlink ref="F7" r:id="rId6" xr:uid="{C93B813D-F075-4A00-A982-6B554F49BA3B}"/>
-    <hyperlink ref="F8" r:id="rId7" xr:uid="{0FEC0EC5-67D9-41E8-BEDC-5BEDC2D89837}"/>
-    <hyperlink ref="F9" r:id="rId8" xr:uid="{48C8F712-E2BC-41F1-8B2B-72D85F9D6B90}"/>
-    <hyperlink ref="F10" r:id="rId9" xr:uid="{995FA3D8-9392-42A9-AC95-9C291EEBE56A}"/>
-    <hyperlink ref="F11" r:id="rId10" xr:uid="{046FB7B3-D2C1-4CB8-A808-DFCB2FC5D899}"/>
-    <hyperlink ref="F12" r:id="rId11" xr:uid="{2DAB4A7B-7DED-4005-9156-B7A7EEC99E4E}"/>
-    <hyperlink ref="F13" r:id="rId12" xr:uid="{992FB07A-C125-4925-AEE6-AA735443E7CA}"/>
-    <hyperlink ref="F14" r:id="rId13" xr:uid="{3DF7F1BB-768C-4D85-B2BA-558643C7932D}"/>
-    <hyperlink ref="F15" r:id="rId14" xr:uid="{3AC2BDDE-EB58-455F-B719-6B3193F71041}"/>
-    <hyperlink ref="F16" r:id="rId15" xr:uid="{366001FA-917B-42BE-A8A6-F0D713A1BBCF}"/>
-    <hyperlink ref="F17" r:id="rId16" xr:uid="{49EE3879-2CF1-44A9-9E46-9D7AB266B951}"/>
-    <hyperlink ref="F18" r:id="rId17" xr:uid="{0FE461E7-2DD0-4D52-B4D6-3F8DD3D9A24E}"/>
-    <hyperlink ref="F19" r:id="rId18" xr:uid="{F7FD7BA7-3C3B-4564-AC8F-245816210EC3}"/>
-    <hyperlink ref="F20" r:id="rId19" xr:uid="{8F147C6F-62EF-4AD5-AD6A-B9C38B69831C}"/>
-    <hyperlink ref="F21" r:id="rId20" xr:uid="{83F9D8C6-3926-4606-806E-988D0D315F4A}"/>
-    <hyperlink ref="F22" r:id="rId21" xr:uid="{FB98054B-C721-4FC7-9CC1-1FF985E8E662}"/>
-    <hyperlink ref="F23" r:id="rId22" xr:uid="{284020E0-DC34-4C0D-900F-42AF08B7573B}"/>
-    <hyperlink ref="F24" r:id="rId23" xr:uid="{76B86F20-DACC-483D-BE57-11F658B648E8}"/>
-    <hyperlink ref="F25" r:id="rId24" xr:uid="{8D809D2C-ED18-4F8B-98CE-CB11E39E4725}"/>
-    <hyperlink ref="F26" r:id="rId25" xr:uid="{6F9B8196-B8D4-477D-85DD-AD787AD4F191}"/>
-    <hyperlink ref="F27" r:id="rId26" xr:uid="{DFEBA645-7268-420C-86DF-30EEB3ADEB12}"/>
-    <hyperlink ref="F28" r:id="rId27" xr:uid="{6FAC3600-2F41-4E46-B741-96060FD74F4C}"/>
-    <hyperlink ref="F29" r:id="rId28" xr:uid="{39A79DEE-BF30-42E9-873F-CCD4DC18C59E}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{C2E11FBC-70C3-4175-B407-3AE3B5AB88B9}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{5D46BCE6-875C-4DD1-A561-F12602AA0818}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{C9298B6A-3400-4298-BFA1-CDF2C509364B}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{BBEFC72C-BD5C-40B9-99D1-E240C18CA4E6}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{63ED79AB-A47C-4E8A-AE04-F860DCF5B935}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{C93B813D-F075-4A00-A982-6B554F49BA3B}"/>
+    <hyperlink ref="E8" r:id="rId7" xr:uid="{0FEC0EC5-67D9-41E8-BEDC-5BEDC2D89837}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{48C8F712-E2BC-41F1-8B2B-72D85F9D6B90}"/>
+    <hyperlink ref="E10" r:id="rId9" xr:uid="{995FA3D8-9392-42A9-AC95-9C291EEBE56A}"/>
+    <hyperlink ref="E11" r:id="rId10" xr:uid="{046FB7B3-D2C1-4CB8-A808-DFCB2FC5D899}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{2DAB4A7B-7DED-4005-9156-B7A7EEC99E4E}"/>
+    <hyperlink ref="E13" r:id="rId12" xr:uid="{992FB07A-C125-4925-AEE6-AA735443E7CA}"/>
+    <hyperlink ref="E14" r:id="rId13" xr:uid="{3DF7F1BB-768C-4D85-B2BA-558643C7932D}"/>
+    <hyperlink ref="E15" r:id="rId14" xr:uid="{3AC2BDDE-EB58-455F-B719-6B3193F71041}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{366001FA-917B-42BE-A8A6-F0D713A1BBCF}"/>
+    <hyperlink ref="E17" r:id="rId16" xr:uid="{49EE3879-2CF1-44A9-9E46-9D7AB266B951}"/>
+    <hyperlink ref="E18" r:id="rId17" xr:uid="{0FE461E7-2DD0-4D52-B4D6-3F8DD3D9A24E}"/>
+    <hyperlink ref="E19" r:id="rId18" xr:uid="{F7FD7BA7-3C3B-4564-AC8F-245816210EC3}"/>
+    <hyperlink ref="E20" r:id="rId19" xr:uid="{8F147C6F-62EF-4AD5-AD6A-B9C38B69831C}"/>
+    <hyperlink ref="E21" r:id="rId20" xr:uid="{83F9D8C6-3926-4606-806E-988D0D315F4A}"/>
+    <hyperlink ref="E22" r:id="rId21" xr:uid="{FB98054B-C721-4FC7-9CC1-1FF985E8E662}"/>
+    <hyperlink ref="E23" r:id="rId22" xr:uid="{284020E0-DC34-4C0D-900F-42AF08B7573B}"/>
+    <hyperlink ref="E24" r:id="rId23" xr:uid="{76B86F20-DACC-483D-BE57-11F658B648E8}"/>
+    <hyperlink ref="E25" r:id="rId24" xr:uid="{8D809D2C-ED18-4F8B-98CE-CB11E39E4725}"/>
+    <hyperlink ref="E26" r:id="rId25" xr:uid="{6F9B8196-B8D4-477D-85DD-AD787AD4F191}"/>
+    <hyperlink ref="E27" r:id="rId26" xr:uid="{DFEBA645-7268-420C-86DF-30EEB3ADEB12}"/>
+    <hyperlink ref="E28" r:id="rId27" xr:uid="{6FAC3600-2F41-4E46-B741-96060FD74F4C}"/>
+    <hyperlink ref="E29" r:id="rId28" xr:uid="{39A79DEE-BF30-42E9-873F-CCD4DC18C59E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2004,50 +1834,50 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17">
       <c r="A1" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>136</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="119">
       <c r="A2" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="136">
       <c r="A3" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="102">
       <c r="A4" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="85">
       <c r="A5" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="51">
       <c r="B6" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2078,197 +1908,197 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>149</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>151</v>
       </c>
       <c r="E1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
         <v>153</v>
-      </c>
-      <c r="B2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C2" t="s">
-        <v>155</v>
       </c>
       <c r="D2">
         <v>2000</v>
       </c>
       <c r="E2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="F2" t="s">
-        <v>157</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D3">
         <v>2005</v>
       </c>
       <c r="E3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="F3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D4">
         <v>2021</v>
       </c>
       <c r="E4" t="s">
+        <v>163</v>
+      </c>
+      <c r="F4" t="s">
+        <v>164</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="F4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C5" t="s">
         <v>168</v>
-      </c>
-      <c r="B5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C5" t="s">
-        <v>170</v>
       </c>
       <c r="D5">
         <v>2022</v>
       </c>
       <c r="E5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="F5" t="s">
-        <v>172</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D6">
         <v>2022</v>
       </c>
       <c r="E6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="F6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" t="s">
         <v>179</v>
-      </c>
-      <c r="B7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C7" t="s">
-        <v>181</v>
       </c>
       <c r="D7">
         <v>2013</v>
       </c>
       <c r="E7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="F7" t="s">
-        <v>183</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D8">
         <v>2019</v>
       </c>
       <c r="E8" t="s">
+        <v>184</v>
+      </c>
+      <c r="F8" t="s">
+        <v>185</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="F8" t="s">
-        <v>187</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D9">
         <v>2022</v>
       </c>
       <c r="E9" t="s">
+        <v>188</v>
+      </c>
+      <c r="F9" t="s">
+        <v>189</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="F9" t="s">
-        <v>191</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2287,19 +2117,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="580faea4-8732-496b-8492-7623c27c33b7" xsi:nil="true"/>
-    <TaxCatchAll xmlns="593d299c-58c4-4c8b-ba27-5f6dc42636e0" xsi:nil="true"/>
-    <Date xmlns="580faea4-8732-496b-8492-7623c27c33b7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="580faea4-8732-496b-8492-7623c27c33b7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5180BD15CBAA94A92C877AD9F3D72BF" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a69df548c6bb87eceb556ed584238c31">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="580faea4-8732-496b-8492-7623c27c33b7" xmlns:ns3="593d299c-58c4-4c8b-ba27-5f6dc42636e0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f2420176949b5530f8fa9defd41a6330" ns2:_="" ns3:_="">
     <xsd:import namespace="580faea4-8732-496b-8492-7623c27c33b7"/>
@@ -2566,7 +2383,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2575,24 +2392,20 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4988D492-DF91-4EF0-B029-7C87F5A8DBFC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="580faea4-8732-496b-8492-7623c27c33b7"/>
-    <ds:schemaRef ds:uri="593d299c-58c4-4c8b-ba27-5f6dc42636e0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="580faea4-8732-496b-8492-7623c27c33b7" xsi:nil="true"/>
+    <TaxCatchAll xmlns="593d299c-58c4-4c8b-ba27-5f6dc42636e0" xsi:nil="true"/>
+    <Date xmlns="580faea4-8732-496b-8492-7623c27c33b7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="580faea4-8732-496b-8492-7623c27c33b7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70D0F36E-C5EC-47D2-8CE4-A1835AD2BC56}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2611,10 +2424,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02015C36-9C29-414C-A5ED-D45EF5FAC00E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4988D492-DF91-4EF0-B029-7C87F5A8DBFC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="580faea4-8732-496b-8492-7623c27c33b7"/>
+    <ds:schemaRef ds:uri="593d299c-58c4-4c8b-ba27-5f6dc42636e0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>